<commit_message>
feat: implement state manager for cycle persistence and add cycle runner batch process
</commit_message>
<xml_diff>
--- a/data/List Akun.xlsx
+++ b/data/List Akun.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="100">
   <si>
     <t>No</t>
   </si>
@@ -70,6 +70,15 @@
     <t>00.czndummy@gmail.com</t>
   </si>
   <si>
+    <t>6.60</t>
+  </si>
+  <si>
+    <t>Asia | 41 Character 5 Star and 26 Lightcone | 6 Team | Rate On | E1 Archeron</t>
+  </si>
+  <si>
+    <t>ikangorengdoang@gmail.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">Asia | Starter TL9 | Mortenax,Firefly,Dahlia,Fugue,Archer,Gilgamesh,Sparkle,Danheng,DrRatio | 3 Golden Companion </t>
   </si>
   <si>
@@ -100,13 +109,13 @@
     <t>asepcihuynoroot@gmail.com</t>
   </si>
   <si>
-    <t>11.80</t>
-  </si>
-  <si>
-    <t>Asia | Ashveil E6 and Robin Summeretto E2 | Danheng,Gilgamesh,Huohuo | 18 Ticket</t>
-  </si>
-  <si>
-    <t>e6ashveilpolos@gmail.com</t>
+    <t>11.70</t>
+  </si>
+  <si>
+    <t>Asia | Evanescia E2,Yaoguang E2,Archer E1 | 3 Team Premium | 3 Lightcone Limited</t>
+  </si>
+  <si>
+    <t>fbiopen086@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">Asia | 40 Character 5 Star and 32 Lightcone| 7 Team | Yaoguang and Cyrene E1 </t>
@@ -118,13 +127,13 @@
     <t>WUWA</t>
   </si>
   <si>
-    <t>1.45</t>
-  </si>
-  <si>
-    <t>SEA | Qingxiao,Aemeath,Cartethyia,Mornye,Sigrika,Rebecca,Lupa,Ciaccona,Chisa,Shorekeeper,Phrolova,Jiyan,Cantarella,Yinlin | 8 Weapon Signature | Mid Explore | EndGame lvl 80</t>
-  </si>
-  <si>
-    <t>fitra.uta22@gmail.com</t>
+    <t>1.70</t>
+  </si>
+  <si>
+    <t>Asia | Lucy E2,Aemeath,Denia,Lynae,Qingxiao,Rebecca,Sigrika,Suisui,Verina | 8 Weapon 5 Star</t>
+  </si>
+  <si>
+    <t>wuwa836@gmail.com</t>
   </si>
   <si>
     <t>CZN</t>
@@ -188,9 +197,6 @@
   </si>
   <si>
     <t>fregilezura@gmail.com edit heidemarie+narja e2</t>
-  </si>
-  <si>
-    <t>ikangorengdoang@gmail.com</t>
   </si>
   <si>
     <t>10.30</t>
@@ -584,7 +590,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="3.13"/>
-    <col customWidth="1" min="4" max="4" width="25.25"/>
+    <col customWidth="1" min="4" max="4" width="72.75"/>
     <col customWidth="1" min="5" max="5" width="38.38"/>
   </cols>
   <sheetData>
@@ -701,11 +707,15 @@
       <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4">
-        <v>6.0</v>
-      </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="C7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
@@ -715,13 +725,13 @@
         <v>6</v>
       </c>
       <c r="C8" s="4">
-        <v>7150.0</v>
+        <v>7120.0</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -732,13 +742,13 @@
         <v>6</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
@@ -749,13 +759,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11">
@@ -765,23 +775,23 @@
         <v>10200.0</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1"/>
       <c r="B12" s="2"/>
       <c r="C12" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
@@ -791,10 +801,10 @@
         <v>12130.0</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
@@ -802,16 +812,16 @@
         <v>1.0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F14" s="2">
         <v>470.0</v>
@@ -829,16 +839,16 @@
         <v>1.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
@@ -846,29 +856,29 @@
         <v>2.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1"/>
       <c r="B18" s="2"/>
       <c r="C18" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19">
@@ -876,16 +886,16 @@
         <v>4.0</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C19" s="5">
         <v>46299.0</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20">
@@ -893,16 +903,16 @@
         <v>5.0</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C20" s="5">
         <v>46300.0</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21">
@@ -910,16 +920,16 @@
         <v>6.0</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22">
@@ -927,16 +937,16 @@
         <v>7.0</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23">
@@ -944,14 +954,14 @@
         <v>8.0</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C23" s="3">
         <v>8.5</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24">
@@ -959,14 +969,14 @@
         <v>9.0</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C24" s="3">
         <v>9.5</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
@@ -974,16 +984,16 @@
         <v>10.0</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26">
@@ -991,16 +1001,16 @@
         <v>11.0</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27">
@@ -1008,16 +1018,16 @@
         <v>12.0</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28">
@@ -1025,16 +1035,16 @@
         <v>13.0</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29">
@@ -1042,10 +1052,10 @@
         <v>14.0</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1055,14 +1065,14 @@
         <v>15.0</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C30" s="3">
         <v>15.5</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31">
@@ -1070,10 +1080,10 @@
         <v>16.0</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -1083,7 +1093,7 @@
         <v>17.0</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C32" s="3">
         <v>17.0</v>
@@ -1096,16 +1106,16 @@
         <v>19.0</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C33" s="5">
         <v>46314.0</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34">
@@ -1113,16 +1123,16 @@
         <v>20.0</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C34" s="5">
         <v>46315.0</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35">
@@ -1130,16 +1140,16 @@
         <v>21.0</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C35" s="5">
         <v>46316.0</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36">
@@ -1147,7 +1157,7 @@
         <v>22.0</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C36" s="3">
         <v>22.0</v>
@@ -1160,16 +1170,16 @@
         <v>23.0</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38">
@@ -1177,16 +1187,16 @@
         <v>24.0</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39">
@@ -1194,10 +1204,10 @@
         <v>25.0</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -1207,13 +1217,13 @@
         <v>26.0</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>18</v>
@@ -1224,16 +1234,16 @@
         <v>27.0</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="42">
@@ -1241,16 +1251,16 @@
         <v>28.0</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43">
@@ -1258,10 +1268,10 @@
         <v>29.0</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -1269,7 +1279,7 @@
     <row r="44">
       <c r="A44" s="6"/>
       <c r="C44" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>

</xml_diff>